<commit_message>
changes to data analysis
</commit_message>
<xml_diff>
--- a/agents_main/FYP Data.xlsx
+++ b/agents_main/FYP Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/someshsahu/Desktop/browser-use-final/agents_main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D55C40CA-2F0C-B24B-BBAB-7FAEFD6A2AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297C554A-2486-5147-A708-06E50FEF395E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="760" windowWidth="27600" windowHeight="17240" firstSheet="3" activeTab="8" xr2:uid="{A5162DA1-3FBB-8147-A438-955B411FAAF2}"/>
+    <workbookView xWindow="1120" yWindow="760" windowWidth="27600" windowHeight="17240" firstSheet="5" activeTab="10" xr2:uid="{A5162DA1-3FBB-8147-A438-955B411FAAF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Layer3 LoginChecker Claude" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,8 @@
     <sheet name="Galxe AlphaHunter Claude" sheetId="7" r:id="rId7"/>
     <sheet name="Galxe AlphaHunter OpenAI" sheetId="8" r:id="rId8"/>
     <sheet name="Layer3 OtherAgents Claude" sheetId="10" r:id="rId9"/>
+    <sheet name="Galxe OtherAgents Claude" sheetId="11" r:id="rId10"/>
+    <sheet name="Galxe OtherAgents OpenAI" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="97">
   <si>
     <t>Tokens</t>
   </si>
@@ -277,13 +279,154 @@
   </si>
   <si>
     <t>QuestCompletionAgent_Tokens</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/sake/GCgn2tpVJy</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/UntitledBank/GCwELtp5Vp</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/TitanNetwork/GCv39tpzhh</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/Nexa/GC4DZt1ygP</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/NFTFeed/GCnr8t1Q6B</t>
+  </si>
+  <si>
+    <t>Follow 3 X Accounts</t>
+  </si>
+  <si>
+    <t>Follow an Account
+Visit 3 sites</t>
+  </si>
+  <si>
+    <t>Follow, Like, Retweet, Visit a site</t>
+  </si>
+  <si>
+    <t>Follow an X account and Follow a page</t>
+  </si>
+  <si>
+    <t>Follow 2 X accounts, Retweet and Quote</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 97397
+TaskVerificationAgent- 43978
+QuestCompletionAgent- 60949</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 104284
+TaskVerificationAgent- 78125
+QuestCompletionAgent- 94244</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 262232
+TaskVerificationAgent- 17715
+QuestCompletionAgent- 16671</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 152096
+TaskVerificationAgent- 69002
+QuestCompletionAgent- 48797</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 276513
+TaskVerificationAgent- 44956
+QuestCompletionAgent- 89769</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 194.97
+TaskVerificationAgent- 176.42
+QuestCompletionAgent- 206.33</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 500.20
+TaskVerificationAgent- 40.38
+QuestCompletionAgent- 36.11</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 279.86
+TaskVerificationAgent- 160.87
+QuestCompletionAgent- 104.54</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 402.11
+TaskVerificationAgent- 82.35
+QuestCompletionAgent- 154.45</t>
+  </si>
+  <si>
+    <t>TaskCompletionAgent- 181.32
+TaskVerificationAgent- 98.78
+QuestCompletionAgent- 132.47</t>
+  </si>
+  <si>
+    <t>Human intervention was required to claim the final reward</t>
+  </si>
+  <si>
+    <t>Human intervention was required to redirect the agent to press the refresh button</t>
+  </si>
+  <si>
+    <t>Human intervention was required to click on the first tweet</t>
+  </si>
+  <si>
+    <t>Tasks Completed</t>
+  </si>
+  <si>
+    <t>Total Tasks</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/Kryll/GCjjYt1fux</t>
+  </si>
+  <si>
+    <t>Like, Retweet, Follow</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/EarnOS/GCKrVt1CUJ</t>
+  </si>
+  <si>
+    <t>Visit 2 websites, Follow 2 X accounts, Follow on Galxe, Retweet a tweet</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/KataraAI/GC2UZt1qLB</t>
+  </si>
+  <si>
+    <t>Follow 2 X Accounts, Like and Retweet a tweet</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/apeironnft/GCMeft1NkX</t>
+  </si>
+  <si>
+    <t>Follow on Galxe and Like a tweet on X`</t>
+  </si>
+  <si>
+    <t>https://app.galxe.com/quest/apeironnft/GC6Npt1rpr</t>
+  </si>
+  <si>
+    <t>Like, Retweet, Follow 2 X accounts</t>
+  </si>
+  <si>
+    <t>Human intervention was unable to break the Agent in loop</t>
+  </si>
+  <si>
+    <t>AI Agent went on and did a completely different quest until human intervention</t>
+  </si>
+  <si>
+    <t>Once again the AI agent went to search for an invalid URL and did not understand the instructions of completing the quest specified in the JSON file</t>
+  </si>
+  <si>
+    <t>Only could complete 1 task which was follow Galxe and then went on to do a different quest</t>
+  </si>
+  <si>
+    <t>Only completed 2 tasks out of 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -301,6 +444,12 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -327,13 +476,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -765,6 +915,565 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BC3762-DCB5-C14C-93FA-9FF1452CA81D}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="47.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="65.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2">
+        <v>97397</v>
+      </c>
+      <c r="E2">
+        <v>43978</v>
+      </c>
+      <c r="F2">
+        <v>60949</v>
+      </c>
+      <c r="G2">
+        <v>181.32</v>
+      </c>
+      <c r="H2">
+        <v>98.78</v>
+      </c>
+      <c r="I2">
+        <v>132.47</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" s="1">
+        <v>3</v>
+      </c>
+      <c r="M2" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3">
+        <v>104284</v>
+      </c>
+      <c r="E3">
+        <v>78125</v>
+      </c>
+      <c r="F3">
+        <v>94244</v>
+      </c>
+      <c r="G3">
+        <v>194.97</v>
+      </c>
+      <c r="H3">
+        <v>176.42</v>
+      </c>
+      <c r="I3">
+        <v>206.33</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="1">
+        <v>3</v>
+      </c>
+      <c r="M3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4">
+        <v>262232</v>
+      </c>
+      <c r="E4">
+        <v>17715</v>
+      </c>
+      <c r="F4">
+        <v>16671</v>
+      </c>
+      <c r="G4">
+        <v>500.2</v>
+      </c>
+      <c r="H4">
+        <v>40.380000000000003</v>
+      </c>
+      <c r="I4">
+        <v>36.11</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L4" s="1">
+        <v>4</v>
+      </c>
+      <c r="M4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5">
+        <v>152096</v>
+      </c>
+      <c r="E5">
+        <v>69002</v>
+      </c>
+      <c r="F5">
+        <v>48797</v>
+      </c>
+      <c r="G5">
+        <v>279.86</v>
+      </c>
+      <c r="H5">
+        <v>160.87</v>
+      </c>
+      <c r="I5">
+        <v>104.54</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L5" s="1">
+        <v>2</v>
+      </c>
+      <c r="M5" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6">
+        <v>276513</v>
+      </c>
+      <c r="E6">
+        <v>44956</v>
+      </c>
+      <c r="F6">
+        <v>89769</v>
+      </c>
+      <c r="G6">
+        <v>402.11</v>
+      </c>
+      <c r="H6">
+        <v>82.35</v>
+      </c>
+      <c r="I6">
+        <v>154.44999999999999</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="1">
+        <v>4</v>
+      </c>
+      <c r="M6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{9502DB97-57BC-AC46-BF2E-FD5B9ACDB338}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{0C5C6A76-227B-8A44-B5F1-34D67BB98E2C}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{22E8456C-BF44-6E47-B3DE-B853CD485E8A}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{1EAADCEF-5640-F949-9329-6543EDF15D9E}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{90DEA0E5-0456-154C-BFD9-851F5EE98A9A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF0CB860-564F-884B-AD65-E53BBBF15D70}">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="45.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="60" customWidth="1"/>
+    <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="L2" s="1">
+        <v>4</v>
+      </c>
+      <c r="M2" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1</v>
+      </c>
+      <c r="M3" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="29" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L6" s="1">
+        <v>2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{AF3D36A1-4DDA-1443-A689-59EA9AA86D02}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{34BDC524-9897-FB41-B950-B41F24092B4D}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{7F48CC5A-88EE-7F40-8E25-9EFBFDDD272C}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{B9AD219D-4DAB-E844-B5CE-6DC1D056A090}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{97C525B6-2D8C-D14A-9B8C-3EC4BE1FD9CD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECCEF1A4-89F8-F743-B601-87F9579C2F5C}">
   <dimension ref="A1:B11"/>

</xml_diff>

<commit_message>
adding in new data
</commit_message>
<xml_diff>
--- a/agents_main/FYP Data.xlsx
+++ b/agents_main/FYP Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/someshsahu/Desktop/browser-use-final/agents_main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37DDAA88-CF86-C541-BB97-138925D99402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD78886F-2D29-E347-BD2D-706A5B66DDEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="500" windowWidth="37200" windowHeight="21100" firstSheet="6" activeTab="8" xr2:uid="{A5162DA1-3FBB-8147-A438-955B411FAAF2}"/>
   </bookViews>
@@ -22,9 +22,11 @@
     <sheet name="Galxe AlphaHunter Claude" sheetId="7" r:id="rId7"/>
     <sheet name="Galxe AlphaHunter OpenAI" sheetId="8" r:id="rId8"/>
     <sheet name="Layer3 OtherAgents Claude" sheetId="10" r:id="rId9"/>
-    <sheet name="Layer3 OtherAgents OpenAI" sheetId="13" r:id="rId10"/>
-    <sheet name="Galxe OtherAgents Claude" sheetId="11" r:id="rId11"/>
-    <sheet name="Galxe OtherAgents OpenAI" sheetId="12" r:id="rId12"/>
+    <sheet name="Layer3 User" sheetId="14" r:id="rId10"/>
+    <sheet name="Layer3 OtherAgents OpenAI" sheetId="13" r:id="rId11"/>
+    <sheet name="Galxe OtherAgents Claude" sheetId="11" r:id="rId12"/>
+    <sheet name="Galxe User" sheetId="15" r:id="rId13"/>
+    <sheet name="Galxe OtherAgents OpenAI" sheetId="12" r:id="rId14"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -47,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="145">
   <si>
     <t>Tokens</t>
   </si>
@@ -519,13 +521,76 @@
   </si>
   <si>
     <t>Could not make the swap on the first quest</t>
+  </si>
+  <si>
+    <t>Total Time</t>
+  </si>
+  <si>
+    <t>Test 1</t>
+  </si>
+  <si>
+    <t>Test 2</t>
+  </si>
+  <si>
+    <t>Test 3</t>
+  </si>
+  <si>
+    <t>Average Total Time</t>
+  </si>
+  <si>
+    <t>Ink Mastery</t>
+  </si>
+  <si>
+    <t>Welcome to Spark</t>
+  </si>
+  <si>
+    <t>Berachain Ecosystem Kyberswap</t>
+  </si>
+  <si>
+    <t>Deposit to Spark Savings Vault</t>
+  </si>
+  <si>
+    <t>Superchain Base</t>
+  </si>
+  <si>
+    <t>Polygon Maxi Stablecoin Enjoyer</t>
+  </si>
+  <si>
+    <t>Berachain Ecosystem Jumper</t>
+  </si>
+  <si>
+    <t>Cubes on Berachain</t>
+  </si>
+  <si>
+    <t>Berachain Ecosystem Welcome</t>
+  </si>
+  <si>
+    <t>Berachain Ecosystem Stargate</t>
+  </si>
+  <si>
+    <t>Quest Name</t>
+  </si>
+  <si>
+    <t>Soneium DeFi: Puffer Finance</t>
+  </si>
+  <si>
+    <t>Soneium DeFi: Yay!</t>
+  </si>
+  <si>
+    <t>Titan Network Community Space #12</t>
+  </si>
+  <si>
+    <t>Nexa Debut Campaign</t>
+  </si>
+  <si>
+    <t>200 $MON from Monad Insider</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -553,6 +618,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -575,7 +646,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -583,6 +654,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1015,15 +1091,308 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE54BD01-0827-F24C-A640-043422199DA0}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2">
+        <v>33.270000000000003</v>
+      </c>
+      <c r="E2">
+        <v>31.65</v>
+      </c>
+      <c r="F2">
+        <v>34.53</v>
+      </c>
+      <c r="G2">
+        <f>AVERAGE(D2:F2)</f>
+        <v>33.15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="43" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>45.49</v>
+      </c>
+      <c r="E3">
+        <v>43.9</v>
+      </c>
+      <c r="F3">
+        <v>44.97</v>
+      </c>
+      <c r="G3" s="7">
+        <f>AVERAGE(D3:F3)</f>
+        <v>44.786666666666669</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4">
+        <v>61.62</v>
+      </c>
+      <c r="E4">
+        <v>62.76</v>
+      </c>
+      <c r="F4">
+        <v>63.22</v>
+      </c>
+      <c r="G4" s="7">
+        <f>AVERAGE(D4:F4)</f>
+        <v>62.533333333333331</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5">
+        <v>73.959999999999994</v>
+      </c>
+      <c r="E5">
+        <v>72.12</v>
+      </c>
+      <c r="F5">
+        <v>75.03</v>
+      </c>
+      <c r="G5" s="7">
+        <f>AVERAGE(D5:F5)</f>
+        <v>73.703333333333333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <v>9.99</v>
+      </c>
+      <c r="E6">
+        <v>8.65</v>
+      </c>
+      <c r="F6">
+        <v>9.34</v>
+      </c>
+      <c r="G6" s="7">
+        <f>AVERAGE(D6:F6)</f>
+        <v>9.3266666666666662</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="57" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7">
+        <v>11.4</v>
+      </c>
+      <c r="E7">
+        <v>11.54</v>
+      </c>
+      <c r="F7">
+        <v>10.98</v>
+      </c>
+      <c r="G7" s="7">
+        <f t="shared" ref="G7:G11" si="0">AVERAGE(D7:F7)</f>
+        <v>11.306666666666667</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8">
+        <v>12.2</v>
+      </c>
+      <c r="E8">
+        <v>11.89</v>
+      </c>
+      <c r="F8">
+        <v>12.46</v>
+      </c>
+      <c r="G8" s="7">
+        <f t="shared" si="0"/>
+        <v>12.183333333333332</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="43" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9">
+        <v>17.04</v>
+      </c>
+      <c r="E9">
+        <v>17.07</v>
+      </c>
+      <c r="F9">
+        <v>16.97</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" si="0"/>
+        <v>17.026666666666667</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="43" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10">
+        <v>12.97</v>
+      </c>
+      <c r="E10">
+        <v>13.22</v>
+      </c>
+      <c r="F10">
+        <v>13.77</v>
+      </c>
+      <c r="G10" s="7">
+        <f t="shared" si="0"/>
+        <v>13.32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="71" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11">
+        <v>60.14</v>
+      </c>
+      <c r="E11">
+        <v>61.28</v>
+      </c>
+      <c r="F11">
+        <v>58.99</v>
+      </c>
+      <c r="G11" s="7">
+        <f t="shared" si="0"/>
+        <v>60.136666666666663</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{1C7EA979-25A6-3E4E-BB1B-252AC940DC35}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{E8414323-D8AA-EE41-A792-7813D2C85DAC}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{2014F19E-07A5-4F46-8A51-544BDA35FC04}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{4BFF3E33-712E-0148-BCFB-4B232F179E1F}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{2EC9558B-724D-DF42-9829-5C8F8E5998A7}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{8DF53925-30E5-3D4F-BAAD-FBC61E38101D}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{55DA8BDC-4CEF-8B47-92B3-34D2A5E27091}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{38AA3C7C-D1B7-D64D-B1BF-9131AEF91DD2}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{6AF72F38-E625-D943-84CF-587EC4603A11}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{ADBAC159-DC3E-7040-B646-40EAA9019AB3}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1858136D-EA47-0046-8F09-232180CBB3FF}">
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5" customWidth="1"/>
-    <col min="3" max="9" width="33.5" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="31.5" hidden="1" customWidth="1"/>
-    <col min="11" max="12" width="31.5" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="33.5" customWidth="1"/>
+    <col min="6" max="6" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="33.5" customWidth="1"/>
+    <col min="10" max="12" width="31.5" customWidth="1"/>
     <col min="13" max="13" width="66" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1075,30 +1444,14 @@
       <c r="B2" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="3">
-        <v>121568</v>
-      </c>
-      <c r="E2" s="3">
-        <v>9382</v>
-      </c>
-      <c r="F2" s="3">
-        <v>11572</v>
-      </c>
-      <c r="G2" s="3">
-        <v>205.54</v>
-      </c>
-      <c r="H2" s="3">
-        <v>35.04</v>
-      </c>
-      <c r="I2" s="3">
-        <v>28.81</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="3">
         <v>0</v>
       </c>
@@ -1116,30 +1469,14 @@
       <c r="B3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3">
-        <v>159090</v>
-      </c>
-      <c r="E3" s="3">
-        <v>9373</v>
-      </c>
-      <c r="F3" s="3">
-        <v>7260</v>
-      </c>
-      <c r="G3" s="3">
-        <v>278.63</v>
-      </c>
-      <c r="H3" s="3">
-        <v>29.05</v>
-      </c>
-      <c r="I3" s="3">
-        <v>22.77</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
       <c r="K3" s="3">
         <v>1</v>
       </c>
@@ -1157,30 +1494,14 @@
       <c r="B4" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="3">
-        <v>148173</v>
-      </c>
-      <c r="E4" s="3">
-        <v>22991</v>
-      </c>
-      <c r="F4" s="3">
-        <v>21156</v>
-      </c>
-      <c r="G4" s="3">
-        <v>276.02999999999997</v>
-      </c>
-      <c r="H4" s="3">
-        <v>56.74</v>
-      </c>
-      <c r="I4" s="3">
-        <v>49.63</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
       <c r="K4" s="3">
         <v>2</v>
       </c>
@@ -1198,30 +1519,14 @@
       <c r="B5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="3">
-        <v>81512</v>
-      </c>
-      <c r="E5" s="3">
-        <v>17442</v>
-      </c>
-      <c r="F5" s="3">
-        <v>7426</v>
-      </c>
-      <c r="G5" s="3">
-        <v>150.80000000000001</v>
-      </c>
-      <c r="H5" s="3">
-        <v>42.69</v>
-      </c>
-      <c r="I5" s="3">
-        <v>18.239999999999998</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>24</v>
-      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
       <c r="K5" s="3">
         <v>1</v>
       </c>
@@ -1239,30 +1544,14 @@
       <c r="B6" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="3">
-        <v>83327</v>
-      </c>
-      <c r="E6" s="3">
-        <v>42940</v>
-      </c>
-      <c r="F6" s="3">
-        <v>11456</v>
-      </c>
-      <c r="G6" s="3">
-        <v>204.4</v>
-      </c>
-      <c r="H6" s="3">
-        <v>99.17</v>
-      </c>
-      <c r="I6" s="3">
-        <v>32.770000000000003</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
       <c r="K6" s="3">
         <v>2</v>
       </c>
@@ -1273,37 +1562,21 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="43" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="3">
-        <v>250412</v>
-      </c>
-      <c r="E7" s="3">
-        <v>21714</v>
-      </c>
-      <c r="F7" s="3">
-        <v>7381</v>
-      </c>
-      <c r="G7" s="3">
-        <v>459.79</v>
-      </c>
-      <c r="H7" s="3">
-        <v>53.33</v>
-      </c>
-      <c r="I7" s="3">
-        <v>19.82</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
       <c r="K7" s="3">
         <v>0</v>
       </c>
@@ -1321,30 +1594,14 @@
       <c r="B8" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="3">
-        <v>111317</v>
-      </c>
-      <c r="E8" s="3">
-        <v>26849</v>
-      </c>
-      <c r="F8" s="3">
-        <v>7442</v>
-      </c>
-      <c r="G8" s="3">
-        <v>178.7</v>
-      </c>
-      <c r="H8" s="3">
-        <v>78.680000000000007</v>
-      </c>
-      <c r="I8" s="3">
-        <v>18.940000000000001</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
       <c r="K8" s="3">
         <v>1</v>
       </c>
@@ -1362,30 +1619,14 @@
       <c r="B9" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="3">
-        <v>92392</v>
-      </c>
-      <c r="E9" s="3">
-        <v>13185</v>
-      </c>
-      <c r="F9" s="3">
-        <v>7428</v>
-      </c>
-      <c r="G9" s="3">
-        <v>156.03</v>
-      </c>
-      <c r="H9" s="3">
-        <v>32.950000000000003</v>
-      </c>
-      <c r="I9" s="3">
-        <v>19.29</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
       <c r="K9" s="3">
         <v>0</v>
       </c>
@@ -1451,9 +1692,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88BC3762-DCB5-C14C-93FA-9FF1452CA81D}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.5" bestFit="1" customWidth="1"/>
@@ -1467,258 +1708,300 @@
     <col min="9" max="9" width="24.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="65.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="65.33203125" customWidth="1"/>
+    <col min="13" max="13" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>97397</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>43978</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>60949</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>181.32</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>98.78</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>132.47</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
+        <f>SUM(H2:J2)</f>
+        <v>412.57000000000005</v>
+      </c>
+      <c r="N2" s="1">
         <v>3</v>
       </c>
-      <c r="M2" s="1">
+      <c r="O2" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>104284</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>78125</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>94244</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>194.97</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>176.42</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>206.33</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="1">
+        <f t="shared" ref="M3:M6" si="0">SUM(H3:J3)</f>
+        <v>577.72</v>
+      </c>
+      <c r="N3" s="1">
         <v>3</v>
       </c>
-      <c r="M3" s="1">
+      <c r="O3" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>262232</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>17715</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>16671</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>500.2</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>40.380000000000003</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>36.11</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
+        <f t="shared" si="0"/>
+        <v>576.69000000000005</v>
+      </c>
+      <c r="N4" s="1">
         <v>4</v>
       </c>
-      <c r="M4" s="1">
+      <c r="O4" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>152096</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>69002</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>48797</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>279.86</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>160.87</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>104.54</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="L5" s="1">
+      <c r="M5" s="1">
+        <f t="shared" si="0"/>
+        <v>545.27</v>
+      </c>
+      <c r="N5" s="1">
         <v>2</v>
       </c>
-      <c r="M5" s="1">
+      <c r="O5" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="85" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>276513</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>44956</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>89769</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>402.11</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>82.35</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>154.44999999999999</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="1">
+        <f t="shared" si="0"/>
+        <v>638.91000000000008</v>
+      </c>
+      <c r="N6" s="1">
         <v>4</v>
       </c>
-      <c r="M6" s="1">
+      <c r="O6" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="L7" s="1"/>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1734,7 +2017,188 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{233D017F-0683-A64A-A555-FD51FF615EBB}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="47.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.5" customWidth="1"/>
+    <col min="3" max="3" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2">
+        <v>53.82</v>
+      </c>
+      <c r="E2">
+        <v>55.79</v>
+      </c>
+      <c r="F2">
+        <v>52.23</v>
+      </c>
+      <c r="G2" s="7">
+        <f>AVERAGE(D2:F2)</f>
+        <v>53.946666666666665</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3">
+        <v>52.44</v>
+      </c>
+      <c r="E3">
+        <v>52.35</v>
+      </c>
+      <c r="F3">
+        <v>53.66</v>
+      </c>
+      <c r="G3" s="7">
+        <f>AVERAGE(D3:F3)</f>
+        <v>52.816666666666663</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4">
+        <v>46.08</v>
+      </c>
+      <c r="E4">
+        <v>46.61</v>
+      </c>
+      <c r="F4">
+        <v>45.89</v>
+      </c>
+      <c r="G4" s="7">
+        <f>AVERAGE(D4:F4)</f>
+        <v>46.193333333333328</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D5">
+        <v>22.28</v>
+      </c>
+      <c r="E5">
+        <v>23.21</v>
+      </c>
+      <c r="F5">
+        <v>22.74</v>
+      </c>
+      <c r="G5" s="7">
+        <f>AVERAGE(D5:F5)</f>
+        <v>22.743333333333336</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6">
+        <v>44.98</v>
+      </c>
+      <c r="E6">
+        <v>44.72</v>
+      </c>
+      <c r="F6">
+        <v>45.05</v>
+      </c>
+      <c r="G6" s="7">
+        <f>AVERAGE(D6:F6)</f>
+        <v>44.916666666666664</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G11" s="7"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{7CC5CC57-38D9-9F44-B54A-05689A5FEE50}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{083E3215-DFB5-5D4C-9DC3-181BDE956BC2}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{F1DD588C-484B-EF49-B2A5-4EB28E7FCECC}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{8A82522C-937D-0345-84F2-6ED7344764BC}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{0563095F-F9B2-BD4E-B624-7CC69908673C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF0CB860-564F-884B-AD65-E53BBBF15D70}">
   <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2698,458 +3162,562 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80ADB110-86FA-7642-8276-6C5B1BD048E0}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.5" customWidth="1"/>
-    <col min="3" max="9" width="33.5" customWidth="1"/>
-    <col min="10" max="12" width="31.5" customWidth="1"/>
-    <col min="13" max="13" width="66" customWidth="1"/>
+    <col min="2" max="2" width="53.33203125" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+    <col min="4" max="10" width="33.5" customWidth="1"/>
+    <col min="11" max="14" width="31.5" customWidth="1"/>
+    <col min="15" max="15" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="57" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="57" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3">
+      <c r="E2" s="3">
         <v>121568</v>
       </c>
-      <c r="E2" s="3">
+      <c r="F2" s="3">
         <v>9382</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="3">
         <v>11572</v>
       </c>
-      <c r="G2" s="3">
+      <c r="H2" s="3">
         <v>205.54</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="3">
         <v>35.04</v>
       </c>
-      <c r="I2" s="3">
+      <c r="J2" s="3">
         <v>28.81</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="K2" s="3">
-        <v>4</v>
       </c>
       <c r="L2" s="3">
         <v>4</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="3">
+        <v>4</v>
+      </c>
+      <c r="N2" s="3">
+        <f>SUM(H2:J2)</f>
+        <v>269.39</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3">
+      <c r="E3" s="3">
         <v>159090</v>
       </c>
-      <c r="E3" s="3">
+      <c r="F3" s="3">
         <v>9373</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="3">
         <v>7260</v>
       </c>
-      <c r="G3" s="3">
+      <c r="H3" s="3">
         <v>278.63</v>
       </c>
-      <c r="H3" s="3">
+      <c r="I3" s="3">
         <v>29.05</v>
       </c>
-      <c r="I3" s="3">
+      <c r="J3" s="3">
         <v>22.77</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="K3" s="3">
-        <v>2</v>
       </c>
       <c r="L3" s="3">
         <v>2</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="3">
+        <v>2</v>
+      </c>
+      <c r="N3" s="3">
+        <f>SUM(H3:J3)</f>
+        <v>330.45</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="57" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="57" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="3">
         <v>148173</v>
       </c>
-      <c r="E4" s="3">
+      <c r="F4" s="3">
         <v>22991</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="3">
         <v>21156</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="3">
         <v>276.02999999999997</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>56.74</v>
       </c>
-      <c r="I4" s="3">
+      <c r="J4" s="3">
         <v>49.63</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="K4" s="3">
-        <v>3</v>
       </c>
       <c r="L4" s="3">
         <v>3</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="M4" s="3">
+        <v>3</v>
+      </c>
+      <c r="N4" s="3">
+        <f t="shared" ref="N4:N10" si="0">SUM(H4:J4)</f>
+        <v>382.4</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="57" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="57" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="3">
         <v>81512</v>
       </c>
-      <c r="E5" s="3">
+      <c r="F5" s="3">
         <v>17442</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="3">
         <v>7426</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>150.80000000000001</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>42.69</v>
       </c>
-      <c r="I5" s="3">
+      <c r="J5" s="3">
         <v>18.239999999999998</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="3">
+      <c r="L5" s="3">
         <v>2</v>
       </c>
-      <c r="L5" s="3">
+      <c r="M5" s="3">
         <v>3</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="N5" s="3">
+        <f>SUM(H5:J5)</f>
+        <v>211.73000000000002</v>
+      </c>
+      <c r="O5" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="3">
         <v>83327</v>
       </c>
-      <c r="E6" s="3">
+      <c r="F6" s="3">
         <v>42940</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>11456</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>204.4</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="3">
         <v>99.17</v>
       </c>
-      <c r="I6" s="3">
+      <c r="J6" s="3">
         <v>32.770000000000003</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="K6" s="3">
-        <v>2</v>
       </c>
       <c r="L6" s="3">
         <v>2</v>
       </c>
-      <c r="M6" s="1"/>
-    </row>
-    <row r="7" spans="1:13" ht="57" x14ac:dyDescent="0.2">
+      <c r="M6" s="3">
+        <v>2</v>
+      </c>
+      <c r="N6" s="3">
+        <f>SUM(H6:J6)</f>
+        <v>336.34</v>
+      </c>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" ht="57" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="3">
         <v>250412</v>
       </c>
-      <c r="E7" s="3">
+      <c r="F7" s="3">
         <v>21714</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="3">
         <v>7381</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="3">
         <v>459.79</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>53.33</v>
       </c>
-      <c r="I7" s="3">
+      <c r="J7" s="3">
         <v>19.82</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="3">
+      <c r="L7" s="3">
         <v>2</v>
       </c>
-      <c r="L7" s="3">
+      <c r="M7" s="3">
         <v>3</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="3">
+        <f>SUM(H7:J7)</f>
+        <v>532.94000000000005</v>
+      </c>
+      <c r="O7" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="3">
         <v>111317</v>
       </c>
-      <c r="E8" s="3">
+      <c r="F8" s="3">
         <v>26849</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="3">
         <v>7442</v>
       </c>
-      <c r="G8" s="3">
+      <c r="H8" s="3">
         <v>178.7</v>
       </c>
-      <c r="H8" s="3">
+      <c r="I8" s="3">
         <v>78.680000000000007</v>
       </c>
-      <c r="I8" s="3">
+      <c r="J8" s="3">
         <v>18.940000000000001</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="K8" s="3">
-        <v>2</v>
       </c>
       <c r="L8" s="3">
         <v>2</v>
       </c>
-      <c r="M8" s="1"/>
-    </row>
-    <row r="9" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+      <c r="M8" s="3">
+        <v>2</v>
+      </c>
+      <c r="N8" s="3">
+        <f t="shared" si="0"/>
+        <v>276.32</v>
+      </c>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="3">
+      <c r="E9" s="3">
         <v>92392</v>
       </c>
-      <c r="E9" s="3">
+      <c r="F9" s="3">
         <v>13185</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="3">
         <v>7428</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="3">
         <v>156.03</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>32.950000000000003</v>
       </c>
-      <c r="I9" s="3">
+      <c r="J9" s="3">
         <v>19.29</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="K9" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="K9" s="3">
-        <v>3</v>
       </c>
       <c r="L9" s="3">
         <v>3</v>
       </c>
-      <c r="M9" s="1"/>
-    </row>
-    <row r="10" spans="1:13" ht="43" x14ac:dyDescent="0.2">
+      <c r="M9" s="3">
+        <v>3</v>
+      </c>
+      <c r="N9" s="3">
+        <f>SUM(H9:J9)</f>
+        <v>208.27</v>
+      </c>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" ht="43" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="3">
         <v>130876</v>
       </c>
-      <c r="E10" s="3">
+      <c r="F10" s="3">
         <v>22103</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="3">
         <v>11675</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H10" s="3">
         <v>180.37</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>55.46</v>
       </c>
-      <c r="I10" s="3">
+      <c r="J10" s="3">
         <v>32.35</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="K10" s="3">
-        <v>3</v>
       </c>
       <c r="L10" s="3">
         <v>3</v>
       </c>
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="1:13" ht="71" x14ac:dyDescent="0.2">
+      <c r="M10" s="3">
+        <v>3</v>
+      </c>
+      <c r="N10" s="3">
+        <f t="shared" si="0"/>
+        <v>268.18</v>
+      </c>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" ht="71" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="3">
+      <c r="E11" s="3">
         <v>330641</v>
       </c>
-      <c r="E11" s="3">
+      <c r="F11" s="3">
         <v>10336</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="3">
         <v>7777</v>
       </c>
-      <c r="G11" s="3">
+      <c r="H11" s="3">
         <v>608.47</v>
       </c>
-      <c r="H11" s="3">
+      <c r="I11" s="3">
         <v>31.26</v>
       </c>
-      <c r="I11" s="3">
+      <c r="J11" s="3">
         <v>18.420000000000002</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="K11" s="3">
-        <v>4</v>
       </c>
       <c r="L11" s="3">
         <v>4</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="M11" s="3">
+        <v>4</v>
+      </c>
+      <c r="N11" s="3">
+        <f>SUM(H11:J11)</f>
+        <v>658.15</v>
+      </c>
+      <c r="O11" s="1" t="s">
         <v>20</v>
       </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N16" s="3"/>
+    </row>
+    <row r="17" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N20" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>